<commit_message>
Fix upload crash on workbooks with cell comments
exceljs fails with "Cannot read properties of undefined (reading 'comments')"
on files containing comments/notes. Strip comment parts before loading,
and remove header comments from the template.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BuXPdNtEaDEJ1PmaiAwWBo
</commit_message>
<xml_diff>
--- a/talon-scorecard/public/Talon_GTM_Tracker_Template.xlsx
+++ b/talon-scorecard/public/Talon_GTM_Tracker_Template.xlsx
@@ -177,36 +177,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Talon</author>
-  </authors>
-  <commentList>
-    <comment ref="J1" authorId="0" shapeId="0">
-      <text>
-        <t>Pick from the dropdown.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Talon</author>
-  </authors>
-  <commentList>
-    <comment ref="A1" authorId="0" shapeId="0">
-      <text>
-        <t>Monday of the week. Oct 19 row is the baseline KT set.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -7762,7 +7732,6 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -8306,7 +8275,6 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Track progress from fixed Oct 21 baseline; weekly sheet holds new numbers
Starting totals (26 registered, 4 active employers, 650 profiles,
8 handoffs, 1 placement) are fixed in config. Weekly rows are added
on top, and cards show progress since Oct 21.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BuXPdNtEaDEJ1PmaiAwWBo
</commit_message>
<xml_diff>
--- a/talon-scorecard/public/Talon_GTM_Tracker_Template.xlsx
+++ b/talon-scorecard/public/Talon_GTM_Tracker_Template.xlsx
@@ -571,7 +571,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Add one new row each Monday before the team meeting, using numbers from the Talon dashboard. Older rows build the trend lines.</t>
+          <t>Enter only what is NEW each week (e.g. 3 new employers), one row per week. Tracking starts Oct 21, 2026 from fixed starting totals: 26 registered employers, 4 active employers, 650 completed profiles, 8 candidate handoffs, 1 placement. The site adds your weekly numbers to these.</t>
         </is>
       </c>
     </row>
@@ -7745,11 +7745,11 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -7760,49 +7760,37 @@
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
-          <t>Registered employers</t>
+          <t>New registered employers</t>
         </is>
       </c>
       <c r="C1" s="4" t="inlineStr">
         <is>
-          <t>Active employers</t>
+          <t>New active employers</t>
         </is>
       </c>
       <c r="D1" s="4" t="inlineStr">
         <is>
-          <t>Completed student profiles</t>
+          <t>New completed student profiles</t>
         </is>
       </c>
       <c r="E1" s="4" t="inlineStr">
         <is>
-          <t>Candidate handoffs</t>
+          <t>New candidate handoffs</t>
         </is>
       </c>
       <c r="F1" s="4" t="inlineStr">
         <is>
-          <t>Placements</t>
+          <t>New placements</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="8" t="n">
-        <v>46314</v>
-      </c>
-      <c r="B2" s="9" t="n">
-        <v>26</v>
-      </c>
-      <c r="C2" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="D2" s="9" t="n">
-        <v>650</v>
-      </c>
-      <c r="E2" s="9" t="n">
-        <v>8</v>
-      </c>
-      <c r="F2" s="9" t="n">
-        <v>1</v>
-      </c>
+      <c r="A2" s="8" t="n"/>
+      <c r="B2" s="9" t="n"/>
+      <c r="C2" s="9" t="n"/>
+      <c r="D2" s="9" t="n"/>
+      <c r="E2" s="9" t="n"/>
+      <c r="F2" s="9" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="8" t="n"/>

</xml_diff>